<commit_message>
PDF knowledge base, group silence, attendance search
</commit_message>
<xml_diff>
--- a/HOSPITALITY MEMBERS.xlsx
+++ b/HOSPITALITY MEMBERS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/341706f11dbb6ad1/Documents/Protocol Bot/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{B8933D2A-CF6E-47BB-B1FC-6E30EEB082BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF83D1CF-B224-476B-9B87-37EDF33BBBA7}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="8_{B8933D2A-CF6E-47BB-B1FC-6E30EEB082BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4B44FD61-B591-4864-9B89-F54EB72FA5D0}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{4C2305D9-A961-4A00-AA72-500382EFDABF}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="160">
   <si>
     <t>NAME</t>
   </si>
@@ -505,6 +505,15 @@
   </si>
   <si>
     <t>@Joyifeee</t>
+  </si>
+  <si>
+    <t>@chubionoja</t>
+  </si>
+  <si>
+    <t>@Onyinye49</t>
+  </si>
+  <si>
+    <t>@Ela033298</t>
   </si>
 </sst>
 </file>
@@ -1555,6 +1564,12 @@
       <c r="E30" t="s">
         <v>98</v>
       </c>
+      <c r="G30" s="3">
+        <v>6534789056</v>
+      </c>
+      <c r="H30" t="s">
+        <v>158</v>
+      </c>
     </row>
     <row r="31" spans="1:8">
       <c r="A31" t="s">
@@ -1708,6 +1723,12 @@
       <c r="E39" t="s">
         <v>92</v>
       </c>
+      <c r="G39" s="3">
+        <v>6179135655</v>
+      </c>
+      <c r="H39" t="s">
+        <v>157</v>
+      </c>
     </row>
     <row r="40" spans="1:8">
       <c r="A40" t="s">
@@ -2217,6 +2238,12 @@
       </c>
       <c r="E66" t="s">
         <v>92</v>
+      </c>
+      <c r="G66" s="3">
+        <v>6462616674</v>
+      </c>
+      <c r="H66" t="s">
+        <v>159</v>
       </c>
     </row>
   </sheetData>

</xml_diff>